<commit_message>
VersiÃ³n 0.4 - Mejoras en header, navegaciÃ³n, scripts de verificaciÃ³n y documentaciÃ³n completa del mÃ³dulo de importaciÃ³n
</commit_message>
<xml_diff>
--- a/services/excel/ARCHIVOS DE PRUEBA/personal RRHH.xlsx
+++ b/services/excel/ARCHIVOS DE PRUEBA/personal RRHH.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Analisa Vaccaro\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA  RRHH\services\excel\ARCHIVOS DE PRUEBA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D8AD224-1420-400C-9ED0-30975EE515D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20508" windowHeight="8064"/>
   </bookViews>
   <sheets>
     <sheet name="Actualizado 07.11.2025" sheetId="3" r:id="rId1"/>
@@ -18,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Actualizado 07.11.2025'!$B$1:$M$196</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2192,7 +2191,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="165" formatCode="&quot;B/.&quot;#,##0.00"/>
@@ -2625,26 +2624,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:M203"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32.85546875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.42578125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" style="1" customWidth="1"/>
-    <col min="9" max="10" width="17.42578125" style="4" customWidth="1"/>
-    <col min="11" max="11" width="52.5703125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="27.7109375" style="13" customWidth="1"/>
-    <col min="13" max="13" width="50.85546875" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="1.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="5.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="25.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.44140625" style="1" customWidth="1"/>
+    <col min="9" max="10" width="17.44140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="52.5546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" style="13" customWidth="1"/>
+    <col min="13" max="13" width="50.88671875" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B1" s="3" t="s">
         <v>146</v>
       </c>
@@ -2680,7 +2679,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" s="8">
         <v>1</v>
       </c>
@@ -2701,7 +2700,7 @@
       </c>
       <c r="H2" s="11">
         <f t="shared" ref="H2:H12" ca="1" si="0">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I2" s="5">
         <f t="shared" ref="I2:I12" ca="1" si="1">DATEDIF(G2, H2, "Y")</f>
@@ -2720,7 +2719,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="8">
         <v>2</v>
       </c>
@@ -2741,7 +2740,7 @@
       </c>
       <c r="H3" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I3" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -2760,7 +2759,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="8">
         <v>3</v>
       </c>
@@ -2781,7 +2780,7 @@
       </c>
       <c r="H4" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I4" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -2800,7 +2799,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="8">
         <v>4</v>
       </c>
@@ -2821,7 +2820,7 @@
       </c>
       <c r="H5" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I5" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -2840,7 +2839,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="8">
         <v>5</v>
       </c>
@@ -2861,11 +2860,11 @@
       </c>
       <c r="H6" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I6" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>622</v>
@@ -2880,7 +2879,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="8">
         <v>6</v>
       </c>
@@ -2901,7 +2900,7 @@
       </c>
       <c r="H7" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I7" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -2920,7 +2919,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="8">
         <v>7</v>
       </c>
@@ -2941,7 +2940,7 @@
       </c>
       <c r="H8" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I8" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -2960,7 +2959,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="8">
         <v>8</v>
       </c>
@@ -2981,7 +2980,7 @@
       </c>
       <c r="H9" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I9" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -3000,7 +2999,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="8">
         <v>9</v>
       </c>
@@ -3021,7 +3020,7 @@
       </c>
       <c r="H10" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I10" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -3040,7 +3039,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" s="8">
         <v>10</v>
       </c>
@@ -3061,11 +3060,11 @@
       </c>
       <c r="H11" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I11" s="5">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>622</v>
@@ -3080,7 +3079,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="8">
         <v>11</v>
       </c>
@@ -3101,7 +3100,7 @@
       </c>
       <c r="H12" s="11">
         <f t="shared" ca="1" si="0"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I12" s="5">
         <f t="shared" ca="1" si="1"/>
@@ -3120,7 +3119,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="8">
         <v>12</v>
       </c>
@@ -3141,7 +3140,7 @@
       </c>
       <c r="H13" s="11">
         <f t="shared" ref="H13:H20" ca="1" si="2">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I13" s="5">
         <f t="shared" ref="I13:I20" ca="1" si="3">DATEDIF(G13, H13, "Y")</f>
@@ -3160,7 +3159,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="8">
         <v>13</v>
       </c>
@@ -3181,7 +3180,7 @@
       </c>
       <c r="H14" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I14" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3200,7 +3199,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" s="8">
         <v>14</v>
       </c>
@@ -3221,7 +3220,7 @@
       </c>
       <c r="H15" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I15" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3240,7 +3239,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="8">
         <v>15</v>
       </c>
@@ -3261,7 +3260,7 @@
       </c>
       <c r="H16" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I16" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3280,7 +3279,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="8">
         <v>16</v>
       </c>
@@ -3301,7 +3300,7 @@
       </c>
       <c r="H17" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I17" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3320,7 +3319,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" s="8">
         <v>17</v>
       </c>
@@ -3341,7 +3340,7 @@
       </c>
       <c r="H18" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I18" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3360,7 +3359,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" s="8">
         <v>18</v>
       </c>
@@ -3381,7 +3380,7 @@
       </c>
       <c r="H19" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I19" s="5">
         <f t="shared" ca="1" si="3"/>
@@ -3400,7 +3399,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" s="8">
         <v>19</v>
       </c>
@@ -3421,11 +3420,11 @@
       </c>
       <c r="H20" s="11">
         <f t="shared" ca="1" si="2"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I20" s="5">
         <f t="shared" ca="1" si="3"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J20" s="5" t="s">
         <v>623</v>
@@ -3440,7 +3439,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" s="8">
         <v>20</v>
       </c>
@@ -3461,7 +3460,7 @@
       </c>
       <c r="H21" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I21" s="5">
         <f t="shared" ref="I21:I41" ca="1" si="4">DATEDIF(G21, H21, "Y")</f>
@@ -3480,7 +3479,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="8">
         <v>21</v>
       </c>
@@ -3501,7 +3500,7 @@
       </c>
       <c r="H22" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I22" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3520,7 +3519,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23" s="8">
         <v>22</v>
       </c>
@@ -3541,7 +3540,7 @@
       </c>
       <c r="H23" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I23" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3560,7 +3559,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B24" s="8">
         <v>23</v>
       </c>
@@ -3581,7 +3580,7 @@
       </c>
       <c r="H24" s="11">
         <f t="shared" ref="H24:H41" ca="1" si="5">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I24" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3600,7 +3599,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B25" s="8">
         <v>24</v>
       </c>
@@ -3621,7 +3620,7 @@
       </c>
       <c r="H25" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I25" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3640,7 +3639,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="8">
         <v>25</v>
       </c>
@@ -3661,7 +3660,7 @@
       </c>
       <c r="H26" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I26" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3680,7 +3679,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" s="8">
         <v>26</v>
       </c>
@@ -3701,7 +3700,7 @@
       </c>
       <c r="H27" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I27" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3720,7 +3719,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28" s="8">
         <v>27</v>
       </c>
@@ -3741,11 +3740,11 @@
       </c>
       <c r="H28" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I28" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>625</v>
@@ -3760,7 +3759,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B29" s="8">
         <v>28</v>
       </c>
@@ -3781,7 +3780,7 @@
       </c>
       <c r="H29" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I29" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3800,7 +3799,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B30" s="8">
         <v>29</v>
       </c>
@@ -3821,7 +3820,7 @@
       </c>
       <c r="H30" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I30" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3840,7 +3839,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B31" s="8">
         <v>30</v>
       </c>
@@ -3861,7 +3860,7 @@
       </c>
       <c r="H31" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I31" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3878,7 +3877,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B32" s="8">
         <v>31</v>
       </c>
@@ -3899,7 +3898,7 @@
       </c>
       <c r="H32" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I32" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3918,7 +3917,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="8">
         <v>32</v>
       </c>
@@ -3939,7 +3938,7 @@
       </c>
       <c r="H33" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I33" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3958,7 +3957,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B34" s="8">
         <v>33</v>
       </c>
@@ -3979,7 +3978,7 @@
       </c>
       <c r="H34" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I34" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -3998,7 +3997,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="8">
         <v>34</v>
       </c>
@@ -4019,7 +4018,7 @@
       </c>
       <c r="H35" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I35" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4038,7 +4037,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B36" s="8">
         <v>35</v>
       </c>
@@ -4059,7 +4058,7 @@
       </c>
       <c r="H36" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I36" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4078,7 +4077,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B37" s="8">
         <v>36</v>
       </c>
@@ -4099,7 +4098,7 @@
       </c>
       <c r="H37" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I37" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4118,7 +4117,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B38" s="8">
         <v>37</v>
       </c>
@@ -4139,7 +4138,7 @@
       </c>
       <c r="H38" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I38" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4158,7 +4157,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B39" s="8">
         <v>38</v>
       </c>
@@ -4179,7 +4178,7 @@
       </c>
       <c r="H39" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I39" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4198,7 +4197,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B40" s="8">
         <v>39</v>
       </c>
@@ -4219,7 +4218,7 @@
       </c>
       <c r="H40" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I40" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4238,7 +4237,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B41" s="8">
         <v>40</v>
       </c>
@@ -4259,7 +4258,7 @@
       </c>
       <c r="H41" s="11">
         <f t="shared" ca="1" si="5"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I41" s="5">
         <f t="shared" ca="1" si="4"/>
@@ -4278,7 +4277,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B42" s="8">
         <v>41</v>
       </c>
@@ -4299,7 +4298,7 @@
       </c>
       <c r="H42" s="11">
         <f t="shared" ref="H42:H46" ca="1" si="6">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I42" s="5">
         <f t="shared" ref="I42:I46" ca="1" si="7">DATEDIF(G42, H42, "Y")</f>
@@ -4316,7 +4315,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B43" s="8">
         <v>42</v>
       </c>
@@ -4337,7 +4336,7 @@
       </c>
       <c r="H43" s="11">
         <f t="shared" ca="1" si="6"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I43" s="5">
         <f t="shared" ca="1" si="7"/>
@@ -4356,7 +4355,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B44" s="8">
         <v>43</v>
       </c>
@@ -4377,7 +4376,7 @@
       </c>
       <c r="H44" s="11">
         <f t="shared" ca="1" si="6"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I44" s="5">
         <f t="shared" ca="1" si="7"/>
@@ -4396,7 +4395,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B45" s="8">
         <v>44</v>
       </c>
@@ -4417,7 +4416,7 @@
       </c>
       <c r="H45" s="11">
         <f t="shared" ca="1" si="6"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I45" s="5">
         <f t="shared" ca="1" si="7"/>
@@ -4436,7 +4435,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B46" s="8">
         <v>45</v>
       </c>
@@ -4457,7 +4456,7 @@
       </c>
       <c r="H46" s="11">
         <f t="shared" ca="1" si="6"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I46" s="5">
         <f t="shared" ca="1" si="7"/>
@@ -4476,7 +4475,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B47" s="8">
         <v>46</v>
       </c>
@@ -4497,7 +4496,7 @@
       </c>
       <c r="H47" s="11">
         <f t="shared" ref="H47:H57" ca="1" si="8">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I47" s="5">
         <f t="shared" ref="I47:I57" ca="1" si="9">DATEDIF(G47, H47, "Y")</f>
@@ -4516,7 +4515,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B48" s="8">
         <v>47</v>
       </c>
@@ -4537,7 +4536,7 @@
       </c>
       <c r="H48" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I48" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4556,7 +4555,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B49" s="8">
         <v>48</v>
       </c>
@@ -4577,11 +4576,11 @@
       </c>
       <c r="H49" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I49" s="5">
         <f t="shared" ca="1" si="9"/>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J49" s="5" t="s">
         <v>622</v>
@@ -4596,7 +4595,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B50" s="8">
         <v>49</v>
       </c>
@@ -4617,7 +4616,7 @@
       </c>
       <c r="H50" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I50" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4636,7 +4635,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B51" s="8">
         <v>50</v>
       </c>
@@ -4657,7 +4656,7 @@
       </c>
       <c r="H51" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I51" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4676,7 +4675,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B52" s="8">
         <v>51</v>
       </c>
@@ -4697,7 +4696,7 @@
       </c>
       <c r="H52" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I52" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4716,7 +4715,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B53" s="8">
         <v>52</v>
       </c>
@@ -4737,7 +4736,7 @@
       </c>
       <c r="H53" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I53" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4756,7 +4755,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B54" s="8">
         <v>53</v>
       </c>
@@ -4777,7 +4776,7 @@
       </c>
       <c r="H54" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I54" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4796,7 +4795,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B55" s="8">
         <v>54</v>
       </c>
@@ -4817,7 +4816,7 @@
       </c>
       <c r="H55" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I55" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4836,7 +4835,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B56" s="8">
         <v>55</v>
       </c>
@@ -4857,7 +4856,7 @@
       </c>
       <c r="H56" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I56" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4876,7 +4875,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B57" s="8">
         <v>56</v>
       </c>
@@ -4897,7 +4896,7 @@
       </c>
       <c r="H57" s="11">
         <f t="shared" ca="1" si="8"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I57" s="5">
         <f t="shared" ca="1" si="9"/>
@@ -4916,7 +4915,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B58" s="8">
         <v>57</v>
       </c>
@@ -4937,7 +4936,7 @@
       </c>
       <c r="H58" s="11">
         <f t="shared" ref="H58:H63" ca="1" si="10">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I58" s="5">
         <f t="shared" ref="I58:I70" ca="1" si="11">DATEDIF(G58, H58, "Y")</f>
@@ -4956,7 +4955,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B59" s="8">
         <v>58</v>
       </c>
@@ -4977,7 +4976,7 @@
       </c>
       <c r="H59" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I59" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -4994,7 +4993,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B60" s="8">
         <v>59</v>
       </c>
@@ -5015,7 +5014,7 @@
       </c>
       <c r="H60" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I60" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5032,7 +5031,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B61" s="8">
         <v>60</v>
       </c>
@@ -5053,7 +5052,7 @@
       </c>
       <c r="H61" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I61" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5070,7 +5069,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B62" s="8">
         <v>61</v>
       </c>
@@ -5091,7 +5090,7 @@
       </c>
       <c r="H62" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I62" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5108,7 +5107,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B63" s="8">
         <v>62</v>
       </c>
@@ -5129,7 +5128,7 @@
       </c>
       <c r="H63" s="11">
         <f t="shared" ca="1" si="10"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I63" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5148,7 +5147,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B64" s="8">
         <v>63</v>
       </c>
@@ -5169,7 +5168,7 @@
       </c>
       <c r="H64" s="11">
         <f t="shared" ref="H64:H70" ca="1" si="12">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I64" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5188,7 +5187,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" s="8">
         <v>64</v>
       </c>
@@ -5209,7 +5208,7 @@
       </c>
       <c r="H65" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I65" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5228,7 +5227,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" s="8">
         <v>65</v>
       </c>
@@ -5249,7 +5248,7 @@
       </c>
       <c r="H66" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I66" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5266,7 +5265,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" s="8">
         <v>66</v>
       </c>
@@ -5287,7 +5286,7 @@
       </c>
       <c r="H67" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I67" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5306,7 +5305,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" s="8">
         <v>67</v>
       </c>
@@ -5327,7 +5326,7 @@
       </c>
       <c r="H68" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I68" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5346,7 +5345,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B69" s="8">
         <v>68</v>
       </c>
@@ -5367,7 +5366,7 @@
       </c>
       <c r="H69" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I69" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5386,7 +5385,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B70" s="8">
         <v>69</v>
       </c>
@@ -5407,7 +5406,7 @@
       </c>
       <c r="H70" s="11">
         <f t="shared" ca="1" si="12"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I70" s="5">
         <f t="shared" ca="1" si="11"/>
@@ -5426,7 +5425,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B71" s="8">
         <v>70</v>
       </c>
@@ -5462,7 +5461,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B72" s="8">
         <v>71</v>
       </c>
@@ -5483,7 +5482,7 @@
       </c>
       <c r="H72" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I72" s="5">
         <f ca="1">DATEDIF(G72, H72, "Y")</f>
@@ -5500,7 +5499,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B73" s="8">
         <v>72</v>
       </c>
@@ -5521,7 +5520,7 @@
       </c>
       <c r="H73" s="11">
         <f t="shared" ref="H73:H79" ca="1" si="13">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I73" s="5">
         <f t="shared" ref="I73:I79" ca="1" si="14">DATEDIF(G73, H73, "Y")</f>
@@ -5540,7 +5539,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B74" s="8">
         <v>73</v>
       </c>
@@ -5561,7 +5560,7 @@
       </c>
       <c r="H74" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I74" s="5">
         <f t="shared" ca="1" si="14"/>
@@ -5578,7 +5577,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" s="8">
         <v>74</v>
       </c>
@@ -5599,7 +5598,7 @@
       </c>
       <c r="H75" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I75" s="5">
         <f t="shared" ca="1" si="14"/>
@@ -5618,7 +5617,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B76" s="8">
         <v>75</v>
       </c>
@@ -5639,7 +5638,7 @@
       </c>
       <c r="H76" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I76" s="5">
         <f ca="1">DATEDIF(G76, H76, "Y")</f>
@@ -5658,7 +5657,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B77" s="8">
         <v>76</v>
       </c>
@@ -5679,7 +5678,7 @@
       </c>
       <c r="H77" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I77" s="5">
         <f t="shared" ca="1" si="14"/>
@@ -5698,7 +5697,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="78" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B78" s="8">
         <v>77</v>
       </c>
@@ -5719,7 +5718,7 @@
       </c>
       <c r="H78" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I78" s="5">
         <f t="shared" ca="1" si="14"/>
@@ -5738,7 +5737,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B79" s="8">
         <v>78</v>
       </c>
@@ -5759,7 +5758,7 @@
       </c>
       <c r="H79" s="11">
         <f t="shared" ca="1" si="13"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I79" s="5">
         <f t="shared" ca="1" si="14"/>
@@ -5778,7 +5777,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="80" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B80" s="8">
         <v>79</v>
       </c>
@@ -5799,7 +5798,7 @@
       </c>
       <c r="H80" s="11">
         <f t="shared" ref="H80:H92" ca="1" si="15">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I80" s="5">
         <f t="shared" ref="I80:I92" ca="1" si="16">DATEDIF(G80, H80, "Y")</f>
@@ -5818,7 +5817,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="81" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B81" s="8">
         <v>80</v>
       </c>
@@ -5839,7 +5838,7 @@
       </c>
       <c r="H81" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I81" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -5858,7 +5857,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="82" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B82" s="8">
         <v>81</v>
       </c>
@@ -5879,7 +5878,7 @@
       </c>
       <c r="H82" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I82" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -5898,7 +5897,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="83" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B83" s="8">
         <v>82</v>
       </c>
@@ -5919,7 +5918,7 @@
       </c>
       <c r="H83" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I83" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -5938,7 +5937,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="84" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B84" s="8">
         <v>83</v>
       </c>
@@ -5959,7 +5958,7 @@
       </c>
       <c r="H84" s="15">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I84" s="16">
         <f t="shared" ca="1" si="16"/>
@@ -5978,7 +5977,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="85" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B85" s="8">
         <v>84</v>
       </c>
@@ -5999,7 +5998,7 @@
       </c>
       <c r="H85" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I85" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6018,7 +6017,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="86" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B86" s="8">
         <v>85</v>
       </c>
@@ -6039,7 +6038,7 @@
       </c>
       <c r="H86" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I86" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6058,7 +6057,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="87" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B87" s="8">
         <v>86</v>
       </c>
@@ -6079,7 +6078,7 @@
       </c>
       <c r="H87" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I87" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6096,7 +6095,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="88" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B88" s="8">
         <v>87</v>
       </c>
@@ -6117,7 +6116,7 @@
       </c>
       <c r="H88" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I88" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6136,7 +6135,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="89" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B89" s="8">
         <v>88</v>
       </c>
@@ -6157,7 +6156,7 @@
       </c>
       <c r="H89" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I89" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6176,7 +6175,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="90" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B90" s="8">
         <v>89</v>
       </c>
@@ -6197,7 +6196,7 @@
       </c>
       <c r="H90" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I90" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6216,7 +6215,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="91" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B91" s="8">
         <v>90</v>
       </c>
@@ -6237,7 +6236,7 @@
       </c>
       <c r="H91" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I91" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6256,7 +6255,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="92" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B92" s="8">
         <v>91</v>
       </c>
@@ -6277,7 +6276,7 @@
       </c>
       <c r="H92" s="11">
         <f t="shared" ca="1" si="15"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I92" s="5">
         <f t="shared" ca="1" si="16"/>
@@ -6296,7 +6295,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="93" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B93" s="8">
         <v>92</v>
       </c>
@@ -6317,7 +6316,7 @@
       </c>
       <c r="H93" s="11">
         <f t="shared" ref="H93:H112" ca="1" si="17">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I93" s="5">
         <f t="shared" ref="I93:I112" ca="1" si="18">DATEDIF(G93, H93, "Y")</f>
@@ -6336,7 +6335,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="94" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B94" s="8">
         <v>93</v>
       </c>
@@ -6357,7 +6356,7 @@
       </c>
       <c r="H94" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I94" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6376,7 +6375,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="95" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B95" s="8">
         <v>94</v>
       </c>
@@ -6397,7 +6396,7 @@
       </c>
       <c r="H95" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I95" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6416,7 +6415,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="96" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B96" s="8">
         <v>95</v>
       </c>
@@ -6437,7 +6436,7 @@
       </c>
       <c r="H96" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I96" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6454,7 +6453,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="97" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B97" s="8">
         <v>96</v>
       </c>
@@ -6475,7 +6474,7 @@
       </c>
       <c r="H97" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I97" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6494,7 +6493,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="98" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B98" s="8">
         <v>97</v>
       </c>
@@ -6515,7 +6514,7 @@
       </c>
       <c r="H98" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I98" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6534,7 +6533,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="99" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B99" s="8">
         <v>98</v>
       </c>
@@ -6555,7 +6554,7 @@
       </c>
       <c r="H99" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I99" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6574,7 +6573,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="100" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B100" s="8">
         <v>99</v>
       </c>
@@ -6595,7 +6594,7 @@
       </c>
       <c r="H100" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I100" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6614,7 +6613,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="101" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B101" s="8">
         <v>100</v>
       </c>
@@ -6635,7 +6634,7 @@
       </c>
       <c r="H101" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I101" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6654,7 +6653,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="102" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B102" s="8">
         <v>101</v>
       </c>
@@ -6675,7 +6674,7 @@
       </c>
       <c r="H102" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I102" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6694,7 +6693,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="103" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B103" s="8">
         <v>102</v>
       </c>
@@ -6715,7 +6714,7 @@
       </c>
       <c r="H103" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I103" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6734,7 +6733,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="104" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B104" s="8">
         <v>103</v>
       </c>
@@ -6755,7 +6754,7 @@
       </c>
       <c r="H104" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I104" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6774,7 +6773,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="105" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B105" s="8">
         <v>104</v>
       </c>
@@ -6795,7 +6794,7 @@
       </c>
       <c r="H105" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I105" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6814,7 +6813,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="106" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B106" s="8">
         <v>105</v>
       </c>
@@ -6835,7 +6834,7 @@
       </c>
       <c r="H106" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I106" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6854,7 +6853,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="107" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B107" s="8">
         <v>106</v>
       </c>
@@ -6875,7 +6874,7 @@
       </c>
       <c r="H107" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I107" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6894,7 +6893,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="108" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B108" s="8">
         <v>107</v>
       </c>
@@ -6915,7 +6914,7 @@
       </c>
       <c r="H108" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I108" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6934,7 +6933,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="109" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B109" s="8">
         <v>108</v>
       </c>
@@ -6955,7 +6954,7 @@
       </c>
       <c r="H109" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I109" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -6974,7 +6973,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="110" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B110" s="8">
         <v>109</v>
       </c>
@@ -6995,7 +6994,7 @@
       </c>
       <c r="H110" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I110" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -7014,7 +7013,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="111" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B111" s="8">
         <v>110</v>
       </c>
@@ -7035,7 +7034,7 @@
       </c>
       <c r="H111" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I111" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -7054,7 +7053,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="112" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B112" s="8">
         <v>111</v>
       </c>
@@ -7075,7 +7074,7 @@
       </c>
       <c r="H112" s="11">
         <f t="shared" ca="1" si="17"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I112" s="5">
         <f t="shared" ca="1" si="18"/>
@@ -7094,7 +7093,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="113" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B113" s="8">
         <v>112</v>
       </c>
@@ -7115,7 +7114,7 @@
       </c>
       <c r="H113" s="11">
         <f t="shared" ref="H113:H119" ca="1" si="19">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I113" s="5">
         <f t="shared" ref="I113:I119" ca="1" si="20">DATEDIF(G113, H113, "Y")</f>
@@ -7134,7 +7133,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="114" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B114" s="8">
         <v>113</v>
       </c>
@@ -7155,7 +7154,7 @@
       </c>
       <c r="H114" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I114" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7174,7 +7173,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="115" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B115" s="8">
         <v>114</v>
       </c>
@@ -7195,7 +7194,7 @@
       </c>
       <c r="H115" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I115" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7214,7 +7213,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="116" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B116" s="8">
         <v>115</v>
       </c>
@@ -7235,7 +7234,7 @@
       </c>
       <c r="H116" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I116" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7254,7 +7253,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="117" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B117" s="8">
         <v>116</v>
       </c>
@@ -7275,7 +7274,7 @@
       </c>
       <c r="H117" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I117" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7294,7 +7293,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="118" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B118" s="8">
         <v>117</v>
       </c>
@@ -7315,7 +7314,7 @@
       </c>
       <c r="H118" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I118" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7334,7 +7333,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="119" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B119" s="8">
         <v>118</v>
       </c>
@@ -7355,7 +7354,7 @@
       </c>
       <c r="H119" s="11">
         <f t="shared" ca="1" si="19"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I119" s="5">
         <f t="shared" ca="1" si="20"/>
@@ -7374,7 +7373,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="120" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B120" s="8">
         <v>119</v>
       </c>
@@ -7395,7 +7394,7 @@
       </c>
       <c r="H120" s="11">
         <f t="shared" ref="H120:H129" ca="1" si="21">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I120" s="5">
         <f t="shared" ref="I120:I129" ca="1" si="22">DATEDIF(G120, H120, "Y")</f>
@@ -7414,7 +7413,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="121" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B121" s="8">
         <v>120</v>
       </c>
@@ -7435,7 +7434,7 @@
       </c>
       <c r="H121" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I121" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7454,7 +7453,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="122" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B122" s="8">
         <v>121</v>
       </c>
@@ -7475,7 +7474,7 @@
       </c>
       <c r="H122" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I122" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7492,7 +7491,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="123" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B123" s="8">
         <v>122</v>
       </c>
@@ -7513,7 +7512,7 @@
       </c>
       <c r="H123" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I123" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7532,7 +7531,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="124" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B124" s="8">
         <v>123</v>
       </c>
@@ -7553,7 +7552,7 @@
       </c>
       <c r="H124" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I124" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7572,7 +7571,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="125" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B125" s="8">
         <v>124</v>
       </c>
@@ -7593,7 +7592,7 @@
       </c>
       <c r="H125" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I125" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7612,7 +7611,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="126" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B126" s="8">
         <v>125</v>
       </c>
@@ -7633,7 +7632,7 @@
       </c>
       <c r="H126" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I126" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7652,7 +7651,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="127" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B127" s="8">
         <v>126</v>
       </c>
@@ -7673,7 +7672,7 @@
       </c>
       <c r="H127" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I127" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7692,7 +7691,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="128" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B128" s="8">
         <v>127</v>
       </c>
@@ -7713,7 +7712,7 @@
       </c>
       <c r="H128" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I128" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7732,7 +7731,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="129" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B129" s="8">
         <v>128</v>
       </c>
@@ -7753,7 +7752,7 @@
       </c>
       <c r="H129" s="11">
         <f t="shared" ca="1" si="21"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I129" s="5">
         <f t="shared" ca="1" si="22"/>
@@ -7772,7 +7771,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="130" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B130" s="8">
         <v>129</v>
       </c>
@@ -7793,7 +7792,7 @@
       </c>
       <c r="H130" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I130" s="5">
         <f ca="1">DATEDIF(G130, H130, "Y")</f>
@@ -7812,7 +7811,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="131" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B131" s="8">
         <v>130</v>
       </c>
@@ -7833,7 +7832,7 @@
       </c>
       <c r="H131" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I131" s="5">
         <f ca="1">DATEDIF(G131, H131, "Y")</f>
@@ -7852,7 +7851,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="132" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B132" s="8">
         <v>131</v>
       </c>
@@ -7873,7 +7872,7 @@
       </c>
       <c r="H132" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I132" s="5">
         <f ca="1">DATEDIF(G132, H132, "Y")</f>
@@ -7892,7 +7891,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="133" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B133" s="8">
         <v>132</v>
       </c>
@@ -7913,7 +7912,7 @@
       </c>
       <c r="H133" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I133" s="5">
         <f ca="1">DATEDIF(G133, H133, "Y")</f>
@@ -7932,7 +7931,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="134" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B134" s="8">
         <v>133</v>
       </c>
@@ -7953,7 +7952,7 @@
       </c>
       <c r="H134" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I134" s="5">
         <f ca="1">DATEDIF(G134, H134, "Y")</f>
@@ -7972,7 +7971,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="135" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B135" s="8">
         <v>134</v>
       </c>
@@ -7993,7 +7992,7 @@
       </c>
       <c r="H135" s="11">
         <f t="shared" ref="H135:H143" ca="1" si="23">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I135" s="5">
         <f t="shared" ref="I135:I143" ca="1" si="24">DATEDIF(G135, H135, "Y")</f>
@@ -8012,7 +8011,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="136" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B136" s="8">
         <v>135</v>
       </c>
@@ -8033,7 +8032,7 @@
       </c>
       <c r="H136" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I136" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8052,7 +8051,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="137" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B137" s="8">
         <v>136</v>
       </c>
@@ -8073,7 +8072,7 @@
       </c>
       <c r="H137" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I137" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8092,7 +8091,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="138" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B138" s="8">
         <v>137</v>
       </c>
@@ -8113,7 +8112,7 @@
       </c>
       <c r="H138" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I138" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8132,7 +8131,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="139" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B139" s="8">
         <v>138</v>
       </c>
@@ -8153,7 +8152,7 @@
       </c>
       <c r="H139" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I139" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8172,7 +8171,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="140" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B140" s="8">
         <v>139</v>
       </c>
@@ -8193,7 +8192,7 @@
       </c>
       <c r="H140" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I140" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8212,7 +8211,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="141" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B141" s="8">
         <v>140</v>
       </c>
@@ -8233,7 +8232,7 @@
       </c>
       <c r="H141" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I141" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8252,7 +8251,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="142" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B142" s="8">
         <v>141</v>
       </c>
@@ -8273,7 +8272,7 @@
       </c>
       <c r="H142" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I142" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8292,7 +8291,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="143" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B143" s="8">
         <v>142</v>
       </c>
@@ -8313,7 +8312,7 @@
       </c>
       <c r="H143" s="11">
         <f t="shared" ca="1" si="23"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I143" s="5">
         <f t="shared" ca="1" si="24"/>
@@ -8332,7 +8331,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="144" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B144" s="8">
         <v>143</v>
       </c>
@@ -8353,7 +8352,7 @@
       </c>
       <c r="H144" s="11">
         <f t="shared" ref="H144:H158" ca="1" si="25">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I144" s="5">
         <f t="shared" ref="I144:I158" ca="1" si="26">DATEDIF(G144, H144, "Y")</f>
@@ -8370,7 +8369,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="145" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B145" s="8">
         <v>144</v>
       </c>
@@ -8391,7 +8390,7 @@
       </c>
       <c r="H145" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I145" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8410,7 +8409,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="146" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B146" s="8">
         <v>145</v>
       </c>
@@ -8431,7 +8430,7 @@
       </c>
       <c r="H146" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I146" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8450,7 +8449,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="147" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B147" s="8">
         <v>146</v>
       </c>
@@ -8471,7 +8470,7 @@
       </c>
       <c r="H147" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I147" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8490,7 +8489,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="148" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B148" s="8">
         <v>147</v>
       </c>
@@ -8511,7 +8510,7 @@
       </c>
       <c r="H148" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I148" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8530,7 +8529,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="149" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B149" s="8">
         <v>148</v>
       </c>
@@ -8551,7 +8550,7 @@
       </c>
       <c r="H149" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I149" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8570,7 +8569,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="150" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B150" s="8">
         <v>149</v>
       </c>
@@ -8591,7 +8590,7 @@
       </c>
       <c r="H150" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I150" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8610,7 +8609,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="151" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B151" s="8">
         <v>150</v>
       </c>
@@ -8631,7 +8630,7 @@
       </c>
       <c r="H151" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I151" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8650,7 +8649,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="152" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B152" s="8">
         <v>151</v>
       </c>
@@ -8671,7 +8670,7 @@
       </c>
       <c r="H152" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I152" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8690,7 +8689,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="153" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B153" s="8">
         <v>152</v>
       </c>
@@ -8711,7 +8710,7 @@
       </c>
       <c r="H153" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I153" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8728,7 +8727,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="154" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B154" s="8">
         <v>153</v>
       </c>
@@ -8749,7 +8748,7 @@
       </c>
       <c r="H154" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I154" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8768,7 +8767,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="155" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B155" s="8">
         <v>154</v>
       </c>
@@ -8789,7 +8788,7 @@
       </c>
       <c r="H155" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I155" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8808,7 +8807,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="156" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B156" s="8">
         <v>155</v>
       </c>
@@ -8829,7 +8828,7 @@
       </c>
       <c r="H156" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I156" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8848,7 +8847,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="157" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B157" s="8">
         <v>156</v>
       </c>
@@ -8869,7 +8868,7 @@
       </c>
       <c r="H157" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I157" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8886,7 +8885,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="158" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B158" s="8">
         <v>157</v>
       </c>
@@ -8907,7 +8906,7 @@
       </c>
       <c r="H158" s="11">
         <f t="shared" ca="1" si="25"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I158" s="5">
         <f t="shared" ca="1" si="26"/>
@@ -8926,7 +8925,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="159" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B159" s="8">
         <v>158</v>
       </c>
@@ -8947,7 +8946,7 @@
       </c>
       <c r="H159" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I159" s="5">
         <f ca="1">DATEDIF(G159, H159, "Y")</f>
@@ -8964,7 +8963,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="160" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B160" s="8">
         <v>159</v>
       </c>
@@ -8985,7 +8984,7 @@
       </c>
       <c r="H160" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I160" s="5">
         <f ca="1">DATEDIF(G160, H160, "Y")</f>
@@ -9004,7 +9003,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="161" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B161" s="8">
         <v>160</v>
       </c>
@@ -9025,7 +9024,7 @@
       </c>
       <c r="H161" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I161" s="5">
         <f ca="1">DATEDIF(G161, H161, "Y")</f>
@@ -9044,7 +9043,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="162" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B162" s="8">
         <v>161</v>
       </c>
@@ -9065,7 +9064,7 @@
       </c>
       <c r="H162" s="11">
         <f t="shared" ref="H162:H168" ca="1" si="27">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I162" s="5">
         <f t="shared" ref="I162:I168" ca="1" si="28">DATEDIF(G162, H162, "Y")</f>
@@ -9084,7 +9083,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="163" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B163" s="8">
         <v>162</v>
       </c>
@@ -9105,7 +9104,7 @@
       </c>
       <c r="H163" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I163" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9124,7 +9123,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="164" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B164" s="8">
         <v>163</v>
       </c>
@@ -9145,7 +9144,7 @@
       </c>
       <c r="H164" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I164" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9164,7 +9163,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="165" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B165" s="8">
         <v>164</v>
       </c>
@@ -9185,7 +9184,7 @@
       </c>
       <c r="H165" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I165" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9204,7 +9203,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="166" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B166" s="8">
         <v>165</v>
       </c>
@@ -9225,7 +9224,7 @@
       </c>
       <c r="H166" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I166" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9244,7 +9243,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="167" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B167" s="8">
         <v>166</v>
       </c>
@@ -9265,7 +9264,7 @@
       </c>
       <c r="H167" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I167" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9284,7 +9283,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="168" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B168" s="8">
         <v>167</v>
       </c>
@@ -9305,7 +9304,7 @@
       </c>
       <c r="H168" s="11">
         <f t="shared" ca="1" si="27"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I168" s="5">
         <f t="shared" ca="1" si="28"/>
@@ -9324,7 +9323,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="169" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B169" s="8">
         <v>168</v>
       </c>
@@ -9345,7 +9344,7 @@
       </c>
       <c r="H169" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I169" s="5">
         <f ca="1">DATEDIF(G169, H169, "Y")</f>
@@ -9364,7 +9363,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="170" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B170" s="8">
         <v>169</v>
       </c>
@@ -9385,7 +9384,7 @@
       </c>
       <c r="H170" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I170" s="5">
         <f ca="1">DATEDIF(G170, H170, "Y")</f>
@@ -9404,7 +9403,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="171" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B171" s="8">
         <v>170</v>
       </c>
@@ -9425,7 +9424,7 @@
       </c>
       <c r="H171" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I171" s="5">
         <f t="shared" ref="I171:I184" ca="1" si="29">DATEDIF(G171, H171, "Y")</f>
@@ -9444,7 +9443,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="172" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B172" s="8">
         <v>171</v>
       </c>
@@ -9465,7 +9464,7 @@
       </c>
       <c r="H172" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I172" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9484,7 +9483,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="173" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B173" s="8">
         <v>172</v>
       </c>
@@ -9505,7 +9504,7 @@
       </c>
       <c r="H173" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I173" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9524,7 +9523,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="174" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B174" s="8">
         <v>173</v>
       </c>
@@ -9563,7 +9562,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="175" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B175" s="8">
         <v>174</v>
       </c>
@@ -9584,7 +9583,7 @@
       </c>
       <c r="H175" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I175" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9603,7 +9602,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="176" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B176" s="8">
         <v>175</v>
       </c>
@@ -9624,7 +9623,7 @@
       </c>
       <c r="H176" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I176" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9643,7 +9642,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="177" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B177" s="8">
         <v>176</v>
       </c>
@@ -9682,7 +9681,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="178" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B178" s="8">
         <v>177</v>
       </c>
@@ -9703,7 +9702,7 @@
       </c>
       <c r="H178" s="11">
         <f t="shared" ref="H178:H184" ca="1" si="30">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I178" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9722,7 +9721,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="179" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B179" s="8">
         <v>178</v>
       </c>
@@ -9743,7 +9742,7 @@
       </c>
       <c r="H179" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I179" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9762,7 +9761,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="180" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B180" s="8">
         <v>179</v>
       </c>
@@ -9783,7 +9782,7 @@
       </c>
       <c r="H180" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I180" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9802,7 +9801,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="181" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B181" s="8">
         <v>180</v>
       </c>
@@ -9823,7 +9822,7 @@
       </c>
       <c r="H181" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I181" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9842,7 +9841,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="182" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B182" s="8">
         <v>181</v>
       </c>
@@ -9863,7 +9862,7 @@
       </c>
       <c r="H182" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I182" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9882,7 +9881,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="183" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B183" s="8">
         <v>182</v>
       </c>
@@ -9903,7 +9902,7 @@
       </c>
       <c r="H183" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I183" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9922,7 +9921,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="184" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B184" s="8">
         <v>183</v>
       </c>
@@ -9943,7 +9942,7 @@
       </c>
       <c r="H184" s="11">
         <f t="shared" ca="1" si="30"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I184" s="5">
         <f t="shared" ca="1" si="29"/>
@@ -9962,7 +9961,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="185" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B185" s="8">
         <v>184</v>
       </c>
@@ -9983,7 +9982,7 @@
       </c>
       <c r="H185" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I185" s="5">
         <f ca="1">DATEDIF(G185, H185, "Y")</f>
@@ -10002,7 +10001,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="186" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B186" s="8">
         <v>185</v>
       </c>
@@ -10023,7 +10022,7 @@
       </c>
       <c r="H186" s="11">
         <f t="shared" ref="H186:H194" ca="1" si="31">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I186" s="5">
         <f t="shared" ref="I186:I194" ca="1" si="32">DATEDIF(G186, H186, "Y")</f>
@@ -10042,7 +10041,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="187" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B187" s="8">
         <v>186</v>
       </c>
@@ -10063,7 +10062,7 @@
       </c>
       <c r="H187" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I187" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10082,7 +10081,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="188" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B188" s="8">
         <v>187</v>
       </c>
@@ -10103,7 +10102,7 @@
       </c>
       <c r="H188" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I188" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10122,7 +10121,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="189" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B189" s="8">
         <v>188</v>
       </c>
@@ -10143,7 +10142,7 @@
       </c>
       <c r="H189" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I189" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10162,7 +10161,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="190" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B190" s="8">
         <v>189</v>
       </c>
@@ -10183,7 +10182,7 @@
       </c>
       <c r="H190" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I190" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10202,7 +10201,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="191" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B191" s="8">
         <v>190</v>
       </c>
@@ -10223,7 +10222,7 @@
       </c>
       <c r="H191" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I191" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10242,7 +10241,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="192" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B192" s="8">
         <v>191</v>
       </c>
@@ -10263,7 +10262,7 @@
       </c>
       <c r="H192" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I192" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10282,7 +10281,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="193" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B193" s="8">
         <v>192</v>
       </c>
@@ -10303,7 +10302,7 @@
       </c>
       <c r="H193" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I193" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10322,7 +10321,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="194" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="194" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B194" s="8">
         <v>193</v>
       </c>
@@ -10343,7 +10342,7 @@
       </c>
       <c r="H194" s="11">
         <f t="shared" ca="1" si="31"/>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I194" s="5">
         <f t="shared" ca="1" si="32"/>
@@ -10362,7 +10361,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="195" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B195" s="8">
         <v>194</v>
       </c>
@@ -10383,7 +10382,7 @@
       </c>
       <c r="H195" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I195" s="5">
         <f ca="1">DATEDIF(G195, H195, "Y")</f>
@@ -10402,7 +10401,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="196" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B196" s="8">
         <v>195</v>
       </c>
@@ -10423,7 +10422,7 @@
       </c>
       <c r="H196" s="11">
         <f ca="1">TODAY()</f>
-        <v>45973</v>
+        <v>45982</v>
       </c>
       <c r="I196" s="5">
         <f ca="1">DATEDIF(G196, H196, "Y")</f>
@@ -10442,31 +10441,31 @@
         <v>361</v>
       </c>
     </row>
-    <row r="197" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C197" s="18"/>
     </row>
-    <row r="199" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C199" s="4"/>
     </row>
-    <row r="200" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="200" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C200" s="4"/>
     </row>
-    <row r="201" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C201" s="4"/>
     </row>
-    <row r="202" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C202" s="4"/>
     </row>
-    <row r="203" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C203" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:M196" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:M196">
+  <autoFilter ref="B1:M196">
+    <sortState ref="B2:M196">
       <sortCondition ref="C2:C196"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:M196">
+  <sortState ref="B2:M196">
     <sortCondition ref="B2:B196"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>